<commit_message>
fix(manutencao): detecção automática de header eliminando colunas Unnamed
</commit_message>
<xml_diff>
--- a/data/Indicadores_manutencao/manutencao.xlsx
+++ b/data/Indicadores_manutencao/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\data\Indicadores_manutencao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF1B296-0C12-40D8-9311-1A7F2F3FC394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35259B3D-A752-499F-BE03-9D8AD406840D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="763" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6764,13 +6764,13 @@
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.21875" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="26.6640625" customWidth="1"/>
-    <col min="5" max="5" width="24.33203125" customWidth="1"/>
-    <col min="6" max="6" width="17.5546875" customWidth="1"/>
-    <col min="7" max="7" width="22.5546875" customWidth="1"/>
-    <col min="8" max="8" width="26" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="13.109375" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" customWidth="1"/>
+    <col min="8" max="8" width="21.109375" customWidth="1"/>
     <col min="9" max="9" width="24.5546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="17" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
insere e atualiza manutencao.xlsx
</commit_message>
<xml_diff>
--- a/data/Indicadores_manutencao/manutencao.xlsx
+++ b/data/Indicadores_manutencao/manutencao.xlsx
@@ -5,10 +5,10 @@
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\data\Indicadores_manutencao\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8e481a7cc57d7010/Área de Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E50FA1-1D4F-4C60-91D0-FB1D715910F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{63E50FA1-1D4F-4C60-91D0-FB1D715910F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F627121E-AFF4-471D-8870-661D9E006ABC}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="763" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6852,7 +6852,7 @@
         <v>6</v>
       </c>
       <c r="D3" s="8">
-        <v>1800</v>
+        <v>1800.05</v>
       </c>
       <c r="E3" s="8">
         <v>2445</v>
@@ -6884,7 +6884,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="8">
-        <v>10476.219999999999</v>
+        <v>10476.200000000001</v>
       </c>
       <c r="E4" s="8">
         <v>460</v>

</xml_diff>

<commit_message>
adiciona arquivo de indicadores INDC. COMERCIAL - ABRIL.docx
</commit_message>
<xml_diff>
--- a/data/Indicadores_manutencao/manutencao.xlsx
+++ b/data/Indicadores_manutencao/manutencao.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\data\Indicadores_manutencao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F63FBA96-B9C8-4318-8219-531E01482539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CEDF75D-6601-42CE-B119-76A2ED61FA31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FA4A0903-8A5F-40BA-8712-46AAF48B56BA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Faturamento Mensal</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>Março</t>
+  </si>
+  <si>
+    <t>Abril</t>
   </si>
 </sst>
 </file>
@@ -507,13 +510,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73D102E3-B151-45B0-865D-C9907B87806D}">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="10" width="12.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -640,6 +643,28 @@
       <c r="J4" s="4">
         <v>10936.22</v>
       </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="5"/>
+      <c r="B5" s="5">
+        <v>2026</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5">
+        <v>0</v>
+      </c>
+      <c r="G5" s="5">
+        <v>0</v>
+      </c>
+      <c r="H5" s="5">
+        <v>0</v>
+      </c>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>